<commit_message>
feat: add managerName field to form and update template handling
</commit_message>
<xml_diff>
--- a/DNTT/Mau_template.xlsx
+++ b/DNTT/Mau_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dsslaptop/Desktop/LTH projects/Tlin/DNTT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654904B0-761A-9E4F-A758-A13451C69C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D55BD5-4734-8D4E-912D-5EA517C7CE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="14840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="14780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ĐNTT" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>CÔNG TY CỔ PHẦN CÔNG NGHỆ FEXI</t>
   </si>
@@ -131,6 +131,9 @@
   </si>
   <si>
     <t>%DIACHI%</t>
+  </si>
+  <si>
+    <t>%TRUONGBOPHAN%</t>
   </si>
 </sst>
 </file>
@@ -288,7 +291,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -350,9 +353,50 @@
     <xf numFmtId="37" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -360,9 +404,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -377,41 +418,6 @@
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -580,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.5" style="4" customWidth="1"/>
@@ -595,28 +601,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
     </row>
     <row r="3" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
@@ -640,16 +646,16 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="39"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" spans="1:8" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6"/>
@@ -657,10 +663,10 @@
       <c r="C6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="29"/>
+      <c r="E6" s="41"/>
       <c r="F6" s="9"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
@@ -678,32 +684,32 @@
       <c r="H7" s="30"/>
     </row>
     <row r="8" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="22" t="s">
+      <c r="B8" s="28"/>
+      <c r="C8" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="24"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
     </row>
     <row r="9" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="33" t="s">
+      <c r="B9" s="28"/>
+      <c r="C9" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
     </row>
     <row r="10" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="30" t="s">
@@ -718,58 +724,58 @@
       <c r="H10" s="30"/>
     </row>
     <row r="11" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="21"/>
-      <c r="C11" s="34" t="s">
+      <c r="B11" s="28"/>
+      <c r="C11" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
     </row>
     <row r="12" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="34" t="s">
+      <c r="B12" s="28"/>
+      <c r="C12" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
     </row>
     <row r="13" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="34" t="s">
+      <c r="B13" s="28"/>
+      <c r="C13" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
     </row>
     <row r="14" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="21"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="37"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="34"/>
     </row>
     <row r="15" spans="1:8" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
@@ -799,10 +805,10 @@
       <c r="A16" s="11">
         <v>1</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="32"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="13" t="s">
         <v>20</v>
       </c>
@@ -820,8 +826,8 @@
     </row>
     <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
-      <c r="B17" s="31"/>
-      <c r="C17" s="32"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
       <c r="D17" s="13"/>
       <c r="E17" s="14"/>
       <c r="F17" s="15"/>
@@ -830,8 +836,8 @@
     </row>
     <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="11"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="32"/>
+      <c r="B18" s="25"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="13"/>
       <c r="E18" s="14"/>
       <c r="F18" s="15"/>
@@ -840,8 +846,8 @@
     </row>
     <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="11"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="32"/>
+      <c r="B19" s="25"/>
+      <c r="C19" s="26"/>
       <c r="D19" s="13"/>
       <c r="E19" s="14"/>
       <c r="F19" s="15"/>
@@ -850,8 +856,8 @@
     </row>
     <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="11"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="32"/>
+      <c r="B20" s="25"/>
+      <c r="C20" s="26"/>
       <c r="D20" s="13"/>
       <c r="E20" s="14"/>
       <c r="F20" s="15"/>
@@ -860,8 +866,8 @@
     </row>
     <row r="21" spans="1:8" ht="45" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="11"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="32"/>
+      <c r="B21" s="25"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="13"/>
       <c r="E21" s="14"/>
       <c r="F21" s="15"/>
@@ -870,10 +876,10 @@
     </row>
     <row r="22" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="18"/>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="40"/>
+      <c r="C22" s="27"/>
       <c r="D22" s="18"/>
       <c r="E22" s="18"/>
       <c r="F22" s="19"/>
@@ -884,18 +890,18 @@
       <c r="H22" s="20"/>
     </row>
     <row r="23" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="39" t="s">
+      <c r="B23" s="22"/>
+      <c r="C23" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D23" s="39"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="39"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
@@ -908,28 +914,36 @@
       <c r="H24" s="1"/>
     </row>
     <row r="25" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="25" t="s">
+      <c r="A25" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="24"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B26" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
+  <mergeCells count="30">
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="A7:H7"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="C9:H9"/>
@@ -943,13 +957,15 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="C14:H14"/>
     <mergeCell ref="B15:C15"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>